<commit_message>
Add TC-BOOKING-010 for CI verification
</commit_message>
<xml_diff>
--- a/TestCases/Booking_TestCase.xlsx
+++ b/TestCases/Booking_TestCase.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAnNganh\SpringMediCareWeb-Selenium-Testing\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{419576DF-126D-4439-8B98-305FF430BCB8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719F8603-28A8-418E-B876-4522D308112A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="86">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -308,6 +308,32 @@
   </si>
   <si>
     <t>Guest chưa đăng nhập vẫn truy cập được trang đặt lịch. Cần bổ sung kiểm tra xác thực trước khi cho phép truy cập chức năng đặt lịch.</t>
+  </si>
+  <si>
+    <t>TC-BOOKING-010</t>
+  </si>
+  <si>
+    <t>Kiểm tra test case mới của chức năng Đặt lịch được thực thi thành công trên Local và GitHub Actions.</t>
+  </si>
+  <si>
+    <t>1: Đăng nhập bằng tài khoản Patient hợp lệ.
+2: Mở trang Bác sĩ và chọn bác sĩ cần đặt lịch.
+3: Mở trang Đặt lịch và kiểm tra các trường cần thiết.
+4: Chọn ngày và giờ hợp lệ, còn trống trong lịch làm việc của bác sĩ.
+5: Nhập ghi chú hợp lệ và nhấn Đặt lịch.
+6: Kiểm tra thông báo thành công và lịch hẹn vừa được tạo với trạng thái pending.
+7: Chạy TC-BOOKING-010 trên môi trường Local và ghi nhận kết quả.
+8: Push source code lên branch CI và kiểm tra GitHub Actions tự động thực thi lại bộ test.
+9: Đối chiếu số lượng test case trước và sau khi bổ sung TC-BOOKING-010.</t>
+  </si>
+  <si>
+    <t>TC-BOOKING-010 thực thi PASS trên Local. Sau khi source code được push lên branch CI, GitHub Actions tự động chạy lại bộ kiểm thử, nhận diện TC-BOOKING-010 và tổng số test case tăng từ 125 lên 126. TC-BOOKING-010 tiếp tục PASS trên môi trường CI.</t>
+  </si>
+  <si>
+    <t>TCBooking10_1, TCBooking10_2</t>
+  </si>
+  <si>
+    <t>TC-BOOKING-010 PASS trên Local. Full suite tăng từ 125 lên 126 test case và đạt 121 PASS, 5 XFAIL. Sau khi push lên branch CI, GitHub Actions tự động chạy lại và thu thập 126 test case.</t>
   </si>
 </sst>
 </file>
@@ -836,7 +862,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AA1000"/>
+  <dimension ref="A1:AA1001"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.44140625" customWidth="1"/>
@@ -1774,20 +1800,36 @@
       <c r="Z25" s="3"/>
       <c r="AA25" s="3"/>
     </row>
-    <row r="26" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
+    <row r="26" spans="1:27" ht="115.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="E26" s="28"/>
+      <c r="F26" s="28"/>
+      <c r="G26" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="H26" s="18">
+        <v>46279</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="J26" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="K26" s="18"/>
+      <c r="L26" s="18"/>
+      <c r="M26" s="22"/>
       <c r="N26" s="3"/>
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
@@ -1805,7 +1847,7 @@
     </row>
     <row r="27" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
-      <c r="B27" s="23"/>
+      <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="3"/>
@@ -1834,7 +1876,7 @@
     </row>
     <row r="28" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
+      <c r="B28" s="23"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
@@ -2070,7 +2112,7 @@
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
-      <c r="F36" s="20"/>
+      <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
@@ -2099,7 +2141,7 @@
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
+      <c r="F37" s="20"/>
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
@@ -30049,20 +30091,50 @@
       <c r="Z1000" s="3"/>
       <c r="AA1000" s="3"/>
     </row>
+    <row r="1001" spans="1:27" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1001" s="3"/>
+      <c r="B1001" s="3"/>
+      <c r="C1001" s="3"/>
+      <c r="D1001" s="3"/>
+      <c r="E1001" s="3"/>
+      <c r="F1001" s="3"/>
+      <c r="G1001" s="3"/>
+      <c r="H1001" s="3"/>
+      <c r="I1001" s="3"/>
+      <c r="J1001" s="3"/>
+      <c r="K1001" s="3"/>
+      <c r="L1001" s="3"/>
+      <c r="M1001" s="3"/>
+      <c r="N1001" s="3"/>
+      <c r="O1001" s="3"/>
+      <c r="P1001" s="3"/>
+      <c r="Q1001" s="3"/>
+      <c r="R1001" s="3"/>
+      <c r="S1001" s="3"/>
+      <c r="T1001" s="3"/>
+      <c r="U1001" s="3"/>
+      <c r="V1001" s="3"/>
+      <c r="W1001" s="3"/>
+      <c r="X1001" s="3"/>
+      <c r="Y1001" s="3"/>
+      <c r="Z1001" s="3"/>
+      <c r="AA1001" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="A14:M14"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D23:F23"/>
+  <mergeCells count="31">
     <mergeCell ref="D25:F25"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="A18:M18"/>
+    <mergeCell ref="D26:F26"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="A21:M21"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="A24:M24"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="A14:M14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="A18:M18"/>
     <mergeCell ref="L9:L10"/>
     <mergeCell ref="M9:M10"/>
     <mergeCell ref="F11:M11"/>
@@ -30093,6 +30165,7 @@
     <hyperlink ref="G23" r:id="rId8" xr:uid="{00000000-0004-0000-0500-000007000000}"/>
     <hyperlink ref="M23" r:id="rId9" xr:uid="{00000000-0004-0000-0500-000008000000}"/>
     <hyperlink ref="G25" r:id="rId10" xr:uid="{00000000-0004-0000-0500-000009000000}"/>
+    <hyperlink ref="G26" r:id="rId11" xr:uid="{00000000-0004-0000-0500-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>